<commit_message>
feat: notifications, partial edit, deployment prep
</commit_message>
<xml_diff>
--- a/docs/Update Spart Part_R11_8-1-2026 (Present).xlsx
+++ b/docs/Update Spart Part_R11_8-1-2026 (Present).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\spare-part-inventory\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B9BC51-BCDA-4E6A-95B8-785ADDE159D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{693832AD-529C-4FD4-8F32-A31B2A436184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{9956B38A-57E8-4DE2-9EC9-8247B93159B1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{9956B38A-57E8-4DE2-9EC9-8247B93159B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="4" r:id="rId1"/>
@@ -19738,12 +19738,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f765a895-6bec-4176-8e9f-fc049974c18c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="105e471e-1176-4611-bc66-d874a636eeaf" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -19988,20 +19990,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f765a895-6bec-4176-8e9f-fc049974c18c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="105e471e-1176-4611-bc66-d874a636eeaf" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{314EB567-AC53-4AC5-9EC5-08CD67B67EBD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{917AA71E-1025-4912-8274-BFB7E3E47ED2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f765a895-6bec-4176-8e9f-fc049974c18c"/>
+    <ds:schemaRef ds:uri="105e471e-1176-4611-bc66-d874a636eeaf"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -20026,12 +20029,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{917AA71E-1025-4912-8274-BFB7E3E47ED2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{314EB567-AC53-4AC5-9EC5-08CD67B67EBD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f765a895-6bec-4176-8e9f-fc049974c18c"/>
-    <ds:schemaRef ds:uri="105e471e-1176-4611-bc66-d874a636eeaf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>